<commit_message>
chequeo economia version 1, ahora debemos agregar los cursos que están hasta ahora (fuera del catalogo VRAI)
</commit_message>
<xml_diff>
--- a/VRAI2026/cursos2026/recopilado_outputs.xlsx
+++ b/VRAI2026/cursos2026/recopilado_outputs.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RepoVRAI\Automate-VRAI-UC\VRAI2026\cursos2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C9EC15-D364-475C-8392-5CAF1630D0F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2EE2B4-D177-4D3D-86C9-7F7F36873919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$601</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4416" uniqueCount="1665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4416" uniqueCount="1664">
   <si>
     <t>RUT UC</t>
   </si>
@@ -5015,9 +5012,6 @@
   </si>
   <si>
     <t xml:space="preserve">CLAS = J:2010 a 2120; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLAS = J:1750 a 1920; </t>
   </si>
 </sst>
 </file>
@@ -5382,6 +5376,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K601"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="7" max="7" width="47.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -10511,7 +10513,7 @@
         <v>852</v>
       </c>
       <c r="G212" t="s">
-        <v>1664</v>
+        <v>182</v>
       </c>
       <c r="H212" t="s">
         <v>82</v>

</xml_diff>